<commit_message>
Sechs Musterfirmen mit vollständiger Dokumentation (Handbuch, 13 Prozesse, Nachweise, Musterauftrag, Auditpläne, Fragen); Auswahl und Wechsel im Testmonat; Kopfzeilen-Erkennung nur am Seitenrand; Rollen je Seite
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fbh8tMSwEdyewM2AJScbNe
</commit_message>
<xml_diff>
--- a/test/testkunde/quellen/QM-Uebersicht.xlsx
+++ b/test/testkunde/quellen/QM-Uebersicht.xlsx
@@ -14,7 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chancen" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schulungsplan" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prüfmittel" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigramm" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maßnahmenplan" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reklamationen" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigramm" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +445,81 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ziele, Lieferanten, Risiken, Chancen, Schulung, Prüfmittel, Organigramm</t>
+          <t>Ziele, Lieferanten, Risiken, Chancen, Schulung, Prüfmittel, Maßnahmen, Reklamationen, Organigramm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Rolle</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Geschäftsführung</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Erika Beispiel, Max Probe</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>QMB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Max Probe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Büro und Einkauf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sabine Büro</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Montage</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tom Monteur (Vorarbeiter), Monteur B, C, D</t>
         </is>
       </c>
     </row>
@@ -458,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +553,16 @@
           <t>Ist 2026</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Verantwortlich</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Termin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -486,19 +572,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>unter 2 %</t>
+          <t>unter 2 % der Aufträge</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>1,4 %</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Max Probe</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Termintreue</t>
+          <t>Termintreue Montage</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,6 +605,16 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>93 %</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Max Probe</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
         </is>
       </c>
     </row>
@@ -520,12 +626,76 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16 h</t>
+          <t>16 h im Jahr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>18 h</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Erika Beispiel</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Wartungsverträge</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>+ 20 Verträge</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+ 14</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Erika Beispiel</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Google-Bewertung</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mindestens 4,7 Sterne</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4,8</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Erika Beispiel</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
         </is>
       </c>
     </row>
@@ -540,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,20 +721,25 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Leistung</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Qualität</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Termintreue</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Preis</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Ergebnis</t>
         </is>
@@ -578,20 +753,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>SHK-Material</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -605,22 +785,123 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Wärmepumpen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>B – Maßnahme</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>B – Maßnahme: Bestellung 6 Wochen vorher</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Elektro Meier</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Elektroanschluss (ausgelagert)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Messtechnik-Hersteller</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kalibrierung (ausgelagert)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entsorgung Becker</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Altkessel, Schrott</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -635,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -659,6 +940,11 @@
           <t>Maßnahme</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Wirksamkeit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -678,7 +964,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Vertretungsplan</t>
+          <t>Vertretungsplan, Patensystem</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>wirksam – Urlaubszeit ohne Terminverschiebung</t>
         </is>
       </c>
     </row>
@@ -701,6 +992,65 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>Lagerbestand</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>teilweise – Termintreue 93 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wissensverlust Rente 2027</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Checklisten, Nachfolger einarbeiten</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>läuft</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Datenverlust Software</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Datensicherung, Rücksicherungstest</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>wirksam (Test 03/2026)</t>
         </is>
       </c>
     </row>
@@ -715,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -734,6 +1084,11 @@
           <t>Maßnahme</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Stand</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -749,6 +1104,33 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Schulung zwei Monteure</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ein Monteur geschult</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wartungsverträge</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>planbarer Umsatz</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>bei jeder Inbetriebnahme anbieten</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+ 14 Verträge</t>
         </is>
       </c>
     </row>
@@ -763,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -782,38 +1164,141 @@
           <t>Termin</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monteur A</t>
+          <t>alle</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wärmepumpen</t>
+          <t>Jahresunterweisung inkl. Qualitätspolitik</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>03/2027</t>
+          <t>12.01.2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Tom Monteur</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wärmepumpen (Hersteller)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>erledigt, wirksam</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Monteur B</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wärmepumpen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>geplant</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Monteur C</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Trinkwasserhygiene</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>11/2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>angemeldet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Max Probe, Tom Monteur</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Erste Hilfe Auffrischung</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>erledigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sabine Büro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Handwerkersoftware</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
@@ -828,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -868,7 +1353,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Druckprüfgerät</t>
+          <t>Druckprüfgerät DP-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -896,6 +1381,23 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>04/2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Drehmomentschlüssel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kalibrierung</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>07/2027</t>
         </is>
       </c>
     </row>
@@ -910,42 +1412,288 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Rolle</t>
+          <t>Nr.</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Person</t>
+          <t>Anlass</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Maßnahme</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Verantwortlich</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Termin</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Wirksamkeit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Geschäftsführung</t>
+          <t>M-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Erika Beispiel, Max Probe</t>
+          <t>Internes Audit VP1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Angebote nachfassen: Erinnerung in der Software</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Max Probe</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>erledigt, Prüfung 12/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>QMB</t>
+          <t>M-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Max Probe</t>
+          <t>Internes Audit VP2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Schulungsnachweis Monteur C nachreichen</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sabine Büro</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reklamation R-2026-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Checkliste Druckprüfung mit Drehmoment und Foto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tom Monteur</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>07.07.2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>wirksam</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>M-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Managementbewertung</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lagerbestand Wärmepumpen aufbauen</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Erika Beispiel</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>31.12.2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>läuft</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Kunde</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Problem</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R-2026-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12.02.2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Privatkunde</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Rechnung doppelt verschickt</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>13.02.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R-2026-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>03.04.2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Wohnbau Musterstadt</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Termin um einen Tag verschoben</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>03.04.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R-2026-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>18.06.2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hausverwaltung Lindenhof</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tropfende Verschraubung</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
         </is>
       </c>
     </row>

</xml_diff>